<commit_message>
Redesigned dashboard with new bronze/copper palette, logo, updated data paths, and payment transaction support
</commit_message>
<xml_diff>
--- a/data/Reports/Customer_details.xlsx
+++ b/data/Reports/Customer_details.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAKSHI\Desktop\Jaiswal_Group\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAKSHI\Downloads\Jaiswal_Group_Report\data\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843069A7-3923-468F-A9A7-9C57AAED2461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57EF5FDC-DCD6-4B81-B7AC-625AF7452CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$113</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="239">
   <si>
     <t>Customer Name</t>
   </si>
@@ -63,12 +63,6 @@
     <t>Adsun Lighting Private Limited West Bengal</t>
   </si>
   <si>
-    <t>Akash Electrics</t>
-  </si>
-  <si>
-    <t>Ali Electric &amp; Electronics</t>
-  </si>
-  <si>
     <t>Allied India Technologies Pvt Ltd</t>
   </si>
   <si>
@@ -105,12 +99,6 @@
     <t>Biplab Kumar Shaw</t>
   </si>
   <si>
-    <t>Biswajeet Electrics(nordusk)</t>
-  </si>
-  <si>
-    <t>Biswajeet Electric (Uncle)</t>
-  </si>
-  <si>
     <t>B. R. TELESERVICES &amp; B.R. WEIGH BRIDGE</t>
   </si>
   <si>
@@ -129,9 +117,6 @@
     <t>Debnath Electrics ( NB)</t>
   </si>
   <si>
-    <t>Dey Electric</t>
-  </si>
-  <si>
     <t>Dinesh Electrics (Dada)</t>
   </si>
   <si>
@@ -144,9 +129,6 @@
     <t>Gupta Electric</t>
   </si>
   <si>
-    <t>Joy Guru Electric&lt;Duttapara&gt;</t>
-  </si>
-  <si>
     <t>Karuna Greentech Pvt Ltd</t>
   </si>
   <si>
@@ -156,9 +138,6 @@
     <t>KLIVIYA ENTERPRISE</t>
   </si>
   <si>
-    <t>Kumar Electric</t>
-  </si>
-  <si>
     <t>Ladhuram Toshniwal &amp; Sons</t>
   </si>
   <si>
@@ -192,15 +171,6 @@
     <t>MAA TARA Electrics(LISTER)</t>
   </si>
   <si>
-    <t>Mahamaya Electrics</t>
-  </si>
-  <si>
-    <t>Mahanta Electric</t>
-  </si>
-  <si>
-    <t>Majumdar Electric</t>
-  </si>
-  <si>
     <t>Majumdar (Panpur)</t>
   </si>
   <si>
@@ -210,15 +180,9 @@
     <t>Manoku &amp; Joyti Electronics</t>
   </si>
   <si>
-    <t>Maruti Electric</t>
-  </si>
-  <si>
     <t>Maya Electrics</t>
   </si>
   <si>
-    <t>Mehir Electric</t>
-  </si>
-  <si>
     <t>Mohanto Electrics</t>
   </si>
   <si>
@@ -246,15 +210,9 @@
     <t>M/S THE TAPAN ELECTRIC(NH)</t>
   </si>
   <si>
-    <t>Naihati Electric</t>
-  </si>
-  <si>
     <t>Neha Electric ltd</t>
   </si>
   <si>
-    <t>New Dey Electrics</t>
-  </si>
-  <si>
     <t>New Garai Elect</t>
   </si>
   <si>
@@ -279,9 +237,6 @@
     <t>PAUL ELECTRIC(Listure)</t>
   </si>
   <si>
-    <t>Paul Electric(NH)</t>
-  </si>
-  <si>
     <t>PAUL ELECTRIC(NORRDUSK)</t>
   </si>
   <si>
@@ -294,9 +249,6 @@
     <t>Quantswift Private Limited</t>
   </si>
   <si>
-    <t>Ramkrishna Electric (BS)</t>
-  </si>
-  <si>
     <t>Roy Electric</t>
   </si>
   <si>
@@ -309,12 +261,6 @@
     <t>Sambhu Electrics</t>
   </si>
   <si>
-    <t>Sarkar Electriccs</t>
-  </si>
-  <si>
-    <t>shaan Electric</t>
-  </si>
-  <si>
     <t>Sharma Electrics</t>
   </si>
   <si>
@@ -333,9 +279,6 @@
     <t>Soma Electric</t>
   </si>
   <si>
-    <t>Sree Guru Electrics</t>
-  </si>
-  <si>
     <t>S.R Electrics</t>
   </si>
   <si>
@@ -387,18 +330,12 @@
     <t>wholesaler</t>
   </si>
   <si>
-    <t>Rinku &amp; Stores</t>
-  </si>
-  <si>
     <t>Nordusk</t>
   </si>
   <si>
     <t>Listure</t>
   </si>
   <si>
-    <t>Rashmi led</t>
-  </si>
-  <si>
     <t>Khaitan</t>
   </si>
   <si>
@@ -642,9 +579,6 @@
     <t>Kanthadhar.</t>
   </si>
   <si>
-    <t>Duttapara</t>
-  </si>
-  <si>
     <t>19BQGPS9536N1ZS</t>
   </si>
   <si>
@@ -696,7 +630,134 @@
     <t>GST NO</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>AKASH ELECTRIC (ICHAPUR)</t>
+  </si>
+  <si>
+    <t>ALI ELECTRIC &amp; ELECTRONICS</t>
+  </si>
+  <si>
+    <t>BEST DEAL MARKETING PVT LTD</t>
+  </si>
+  <si>
+    <t>19AACCB3593N1Z5</t>
+  </si>
+  <si>
+    <t>4A, 2ND, SWAIKA CENTRE, POLLOCK STREET, DALHOUSHI, Kolkata, West Bengal, 700001</t>
+  </si>
+  <si>
+    <t>BISWADIP ELECTRIC (Uncle)</t>
+  </si>
+  <si>
+    <t>BISWJEET  ELECTRIC(nordusk)</t>
+  </si>
+  <si>
+    <t>Cash Sale</t>
+  </si>
+  <si>
+    <t>DEY ELECTRICALS</t>
+  </si>
+  <si>
+    <t>19CECPD5261C1ZW</t>
+  </si>
+  <si>
+    <t>102/7, MAA ANNAPURNA APARTMENT, CHANDRAPALLY, New Barrackpur, North Twenty Four Parganas, West Bengal</t>
+  </si>
+  <si>
+    <t>Dey Electric NH</t>
+  </si>
+  <si>
+    <t>JOY GURU ELECTRIC(Duttapara)</t>
+  </si>
+  <si>
+    <t>KUMAR ELECTRIC (BKP)</t>
+  </si>
+  <si>
+    <t>MAA SARADA ELECTRIC</t>
+  </si>
+  <si>
+    <t>19AVOPS7153D2Z2</t>
+  </si>
+  <si>
+    <t>52/424, RN AVENUE, Patulia, North Twenty Four Parganas, West Bengal</t>
+  </si>
+  <si>
+    <t>MAJUMDER ELECTRIC</t>
+  </si>
+  <si>
+    <t>MARUTI ELECTRIC</t>
+  </si>
+  <si>
+    <t>Ganeshpur, Sewli Telinipara, Debpukur, Kolkata, Teleni
+Para, West Bengal 700121</t>
+  </si>
+  <si>
+    <t>MEHIR ELECTRIC</t>
+  </si>
+  <si>
+    <t>MOHANTO  ELECTRIC</t>
+  </si>
+  <si>
+    <t>NAIHATI ELECTRIC</t>
+  </si>
+  <si>
+    <t>19AMAPS6939A1ZX</t>
+  </si>
+  <si>
+    <t>No.49, G.G.ROAD, GORIFA, 24 PGS. NORTH, KOLKATA, North Twenty Four Parganas, West Bengal</t>
+  </si>
+  <si>
+    <t>PAUL ELECTRIC(NH)</t>
+  </si>
+  <si>
+    <t>RAMKRISHNA ELECTRIC (BARASAT)</t>
+  </si>
+  <si>
+    <t>Rinku &amp;stors</t>
+  </si>
+  <si>
+    <t>R.J. ENTERPRISE</t>
+  </si>
+  <si>
+    <t>19AAXFR8411K1ZD</t>
+  </si>
+  <si>
+    <t>176/2/2, sundia village Road, NORTH 24 PARGANAS, North 24 Parganas, West Bengal, 743126</t>
+  </si>
+  <si>
+    <t>SAI BABA ELECTRICALS &amp; INTERIOR DECORATION</t>
+  </si>
+  <si>
+    <t>19CQLPD3943A1Z1</t>
+  </si>
+  <si>
+    <t>140, B.T Road, Kolkata, North Twenty Four Parganas, West Bengal</t>
+  </si>
+  <si>
+    <t>SARKAR ELECTRICS</t>
+  </si>
+  <si>
+    <t>SHAAN  ELECTRIC</t>
+  </si>
+  <si>
+    <t>SREE GURU ELECTRIC(8697543747)</t>
+  </si>
+  <si>
+    <t>SARADA PALLY (AMTALA) DUTTAPUKUR,</t>
+  </si>
+  <si>
+    <t>THIRTYNINE ENTERPRISE(MAHAMAYA  ELECTRIC)</t>
+  </si>
+  <si>
+    <t>19DWMPS9414R1Z7</t>
+  </si>
+  <si>
+    <t>127, R.N.TAGORE ROAD, KOLKATA, North 24 Parganas, West Bengal, 700109</t>
+  </si>
+  <si>
+    <t>khaitan</t>
+  </si>
+  <si>
+    <t>Rashmi LED</t>
   </si>
 </sst>
 </file>
@@ -720,7 +781,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -730,12 +791,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -767,11 +822,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1052,16 +1112,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G108"/>
+  <dimension ref="A1:G113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.140625" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="49.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.85546875" customWidth="1"/>
     <col min="6" max="6" width="18.5703125" customWidth="1"/>
-    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="7" max="7" width="71.85546875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1078,12 +1138,12 @@
         <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>217</v>
+        <v>195</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1095,2071 +1155,2218 @@
         <v>31656</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>120</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>196</v>
       </c>
       <c r="B3">
-        <v>1605</v>
+        <v>18452</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>116</v>
-      </c>
-      <c r="G3" t="s">
-        <v>218</v>
+        <v>96</v>
+      </c>
+      <c r="F3">
+        <v>6291833527</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>197</v>
       </c>
       <c r="B4">
-        <v>9608</v>
+        <v>12928</v>
       </c>
       <c r="C4" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D4" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="F4">
         <v>7003660445</v>
       </c>
-      <c r="G4" t="s">
-        <v>121</v>
+      <c r="G4" s="3" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="E5" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>3283</v>
       </c>
       <c r="C6" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F6">
         <v>9681179458</v>
       </c>
-      <c r="G6" t="s">
-        <v>123</v>
+      <c r="G6" s="3" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>829</v>
       </c>
       <c r="C7" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D7" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F7">
         <v>7439400145</v>
       </c>
-      <c r="G7" t="s">
-        <v>124</v>
+      <c r="G7" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>402</v>
       </c>
       <c r="C8" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D8" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F8">
         <v>8240088104</v>
       </c>
-      <c r="G8" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G8" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B9">
-        <v>287839</v>
+        <v>198839</v>
       </c>
       <c r="C9" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D9" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="F9">
         <v>9143529316</v>
       </c>
-      <c r="G9" t="s">
-        <v>127</v>
+      <c r="G9" s="3" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>13457</v>
       </c>
       <c r="C10" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D10" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F10">
         <v>6291299792</v>
       </c>
-      <c r="G10" t="s">
-        <v>125</v>
+      <c r="G10" s="3" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>11789</v>
       </c>
       <c r="C11" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D11" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="F11">
         <v>6291162829</v>
       </c>
-      <c r="G11" t="s">
-        <v>128</v>
+      <c r="G11" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12">
         <v>986</v>
       </c>
       <c r="C12" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D12" t="s">
-        <v>116</v>
-      </c>
-      <c r="G12" t="s">
-        <v>129</v>
+        <v>96</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B13">
         <v>153</v>
       </c>
       <c r="C13" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D13" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F13">
         <v>9830293265</v>
       </c>
-      <c r="G13" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G13" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>198</v>
       </c>
       <c r="B14">
-        <v>7705</v>
+        <v>0</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D14" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="E14" t="s">
+        <v>199</v>
       </c>
       <c r="F14">
-        <v>9831266412</v>
-      </c>
-      <c r="G14" t="s">
-        <v>131</v>
+        <v>9830070876</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B15">
-        <v>8020</v>
+        <v>7705</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="F15">
+        <v>9831266412</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B16">
-        <v>2956</v>
+        <v>8020</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D16" t="s">
-        <v>117</v>
-      </c>
-      <c r="G16" t="s">
-        <v>132</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B17">
-        <v>2062</v>
+        <v>2956</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D17" t="s">
-        <v>117</v>
-      </c>
-      <c r="F17">
-        <v>9477640704</v>
-      </c>
-      <c r="G17" t="s">
-        <v>133</v>
+        <v>97</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>201</v>
       </c>
       <c r="B18">
         <v>250</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D18" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="F18">
         <v>8820966667</v>
       </c>
-      <c r="G18" t="s">
-        <v>134</v>
+      <c r="G18" s="3" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>202</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>2062</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D19" t="s">
-        <v>117</v>
-      </c>
-      <c r="E19" t="s">
-        <v>135</v>
+        <v>97</v>
       </c>
       <c r="F19">
-        <v>9831058305</v>
-      </c>
-      <c r="G19" t="s">
-        <v>136</v>
+        <v>9477640704</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B20">
-        <v>15994</v>
+        <v>0</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D20" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="E20" t="s">
-        <v>137</v>
-      </c>
-      <c r="G20" t="s">
-        <v>138</v>
+        <v>114</v>
+      </c>
+      <c r="F20">
+        <v>9831058305</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B21">
-        <v>14469</v>
+        <v>15994</v>
       </c>
       <c r="C21" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D21" t="s">
+        <v>96</v>
+      </c>
+      <c r="E21" t="s">
         <v>116</v>
       </c>
-      <c r="G21" t="s">
-        <v>139</v>
+      <c r="G21" s="3" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>203</v>
       </c>
       <c r="B22">
-        <v>14353</v>
+        <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D22" t="s">
-        <v>116</v>
-      </c>
-      <c r="F22">
-        <v>8582829034</v>
-      </c>
-      <c r="G22" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B23">
-        <v>6027</v>
+        <v>13584</v>
       </c>
       <c r="C23" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D23" t="s">
-        <v>116</v>
-      </c>
-      <c r="G23" t="s">
-        <v>129</v>
+        <v>96</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B24">
-        <v>10740</v>
+        <v>14353</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D24" t="s">
-        <v>117</v>
-      </c>
-      <c r="G24" t="s">
-        <v>141</v>
+        <v>96</v>
+      </c>
+      <c r="F24">
+        <v>8582829034</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B25">
-        <v>150</v>
+        <v>6027</v>
       </c>
       <c r="C25" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D25" t="s">
-        <v>116</v>
-      </c>
-      <c r="G25" t="s">
-        <v>142</v>
+        <v>96</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B26">
-        <v>3000</v>
+        <v>9240</v>
       </c>
       <c r="C26" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D26" t="s">
-        <v>117</v>
-      </c>
-      <c r="G26" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+        <v>97</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>31</v>
+        <v>204</v>
       </c>
       <c r="B27">
-        <v>2390</v>
+        <v>15250</v>
       </c>
       <c r="C27" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D27" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="E27" t="s">
-        <v>144</v>
+        <v>205</v>
       </c>
       <c r="F27">
-        <v>7278552805</v>
-      </c>
-      <c r="G27" t="s">
-        <v>145</v>
+        <v>9038901683</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>32</v>
+        <v>207</v>
       </c>
       <c r="B28">
-        <v>60680</v>
+        <v>150</v>
       </c>
       <c r="C28" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D28" t="s">
-        <v>116</v>
-      </c>
-      <c r="F28">
-        <v>9330088639</v>
-      </c>
-      <c r="G28" t="s">
-        <v>146</v>
+        <v>96</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B29">
-        <v>3900</v>
+        <v>3000</v>
       </c>
       <c r="C29" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D29" t="s">
-        <v>116</v>
-      </c>
-      <c r="F29">
-        <v>9831975376</v>
-      </c>
-      <c r="G29" t="s">
+        <v>97</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30">
+        <v>2390</v>
+      </c>
+      <c r="C30" t="s">
+        <v>94</v>
+      </c>
+      <c r="D30" t="s">
+        <v>96</v>
+      </c>
+      <c r="E30" t="s">
+        <v>123</v>
+      </c>
+      <c r="F30">
+        <v>7278552805</v>
+      </c>
+      <c r="G30" s="3" t="s">
         <v>124</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30">
-        <v>2980</v>
-      </c>
-      <c r="C30" t="s">
-        <v>113</v>
-      </c>
-      <c r="D30" t="s">
-        <v>116</v>
-      </c>
-      <c r="F30">
-        <v>9735759791</v>
-      </c>
-      <c r="G30" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B31">
-        <v>0</v>
+        <v>60680</v>
       </c>
       <c r="C31" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="D31" t="s">
-        <v>116</v>
-      </c>
-      <c r="E31" t="s">
-        <v>148</v>
+        <v>96</v>
       </c>
       <c r="F31">
-        <v>9830045014</v>
+        <v>9330088639</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B32">
-        <v>11415</v>
+        <v>3900</v>
       </c>
       <c r="C32" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D32" t="s">
-        <v>116</v>
-      </c>
-      <c r="G32" t="s">
-        <v>129</v>
+        <v>96</v>
+      </c>
+      <c r="F32">
+        <v>9831975376</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>208</v>
       </c>
       <c r="B33">
-        <v>186580.06</v>
+        <v>2980</v>
       </c>
       <c r="C33" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D33" t="s">
-        <v>117</v>
-      </c>
-      <c r="E33" t="s">
-        <v>149</v>
+        <v>96</v>
       </c>
       <c r="F33">
-        <v>9038977095</v>
-      </c>
-      <c r="G33" t="s">
-        <v>150</v>
+        <v>9735759791</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="B34">
-        <v>35194</v>
+        <v>0</v>
       </c>
       <c r="C34" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D34" t="s">
-        <v>116</v>
-      </c>
-      <c r="G34" t="s">
-        <v>151</v>
+        <v>96</v>
+      </c>
+      <c r="E34" t="s">
+        <v>127</v>
+      </c>
+      <c r="F34">
+        <v>9830045014</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B35">
-        <v>0</v>
+        <v>11415</v>
       </c>
       <c r="C35" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="D35" t="s">
-        <v>118</v>
-      </c>
-      <c r="E35" t="s">
-        <v>152</v>
-      </c>
-      <c r="F35">
-        <v>9830055058</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="B36">
-        <v>24595</v>
+        <v>222168.06</v>
       </c>
       <c r="C36" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D36" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="E36" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="F36">
-        <v>8981490138</v>
-      </c>
-      <c r="G36" t="s">
-        <v>154</v>
+        <v>9038977095</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>209</v>
       </c>
       <c r="B37">
-        <v>9140</v>
+        <v>35119</v>
       </c>
       <c r="C37" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D37" t="s">
-        <v>116</v>
-      </c>
-      <c r="F37">
-        <v>9471677578</v>
-      </c>
-      <c r="G37" t="s">
-        <v>151</v>
+        <v>96</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B38">
-        <v>36892</v>
+        <v>0</v>
       </c>
       <c r="C38" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D38" t="s">
-        <v>117</v>
+        <v>238</v>
       </c>
       <c r="E38" t="s">
-        <v>155</v>
+        <v>131</v>
       </c>
       <c r="F38">
-        <v>9830836296</v>
-      </c>
-      <c r="G38" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+        <v>9830055058</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B39">
-        <v>3850</v>
+        <v>24595</v>
       </c>
       <c r="C39" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D39" t="s">
-        <v>116</v>
+        <v>97</v>
+      </c>
+      <c r="E39" t="s">
+        <v>132</v>
       </c>
       <c r="F39">
-        <v>8961765331</v>
-      </c>
-      <c r="G39" t="s">
-        <v>157</v>
+        <v>8981490138</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="B40">
-        <v>14772</v>
+        <v>9140</v>
       </c>
       <c r="C40" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D40" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="F40">
-        <v>9903843406</v>
-      </c>
-      <c r="G40" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>45</v>
+        <v>9471677578</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>35</v>
       </c>
       <c r="B41">
-        <v>0</v>
+        <v>40117</v>
       </c>
       <c r="C41" t="s">
-        <v>113</v>
-      </c>
-      <c r="G41" t="s">
-        <v>159</v>
+        <v>94</v>
+      </c>
+      <c r="D41" t="s">
+        <v>97</v>
+      </c>
+      <c r="E41" t="s">
+        <v>134</v>
+      </c>
+      <c r="F41">
+        <v>9830836296</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B42">
-        <v>859</v>
+        <v>2410</v>
       </c>
       <c r="C42" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D42" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F42">
-        <v>9163055089</v>
-      </c>
-      <c r="G42" t="s">
-        <v>125</v>
+        <v>8961765331</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B43">
-        <v>3528</v>
+        <v>9683</v>
       </c>
       <c r="C43" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D43" t="s">
-        <v>117</v>
-      </c>
-      <c r="G43" t="s">
-        <v>160</v>
+        <v>97</v>
+      </c>
+      <c r="F43">
+        <v>9903843406</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B44">
-        <v>10675</v>
+        <v>0</v>
       </c>
       <c r="C44" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D44" t="s">
-        <v>116</v>
-      </c>
-      <c r="E44" t="s">
-        <v>161</v>
-      </c>
-      <c r="F44">
-        <v>9330817822</v>
-      </c>
-      <c r="G44" t="s">
-        <v>162</v>
+        <v>96</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B45">
-        <v>19224</v>
+        <v>859</v>
       </c>
       <c r="C45" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D45" t="s">
-        <v>117</v>
-      </c>
-      <c r="G45" t="s">
-        <v>163</v>
+        <v>96</v>
+      </c>
+      <c r="F45">
+        <v>9163055089</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B46">
-        <v>39098</v>
+        <v>3528</v>
       </c>
       <c r="C46" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D46" t="s">
-        <v>117</v>
+        <v>97</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>51</v>
+        <v>210</v>
       </c>
       <c r="B47">
-        <v>1409</v>
+        <v>18800</v>
       </c>
       <c r="C47" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D47" t="s">
-        <v>116</v>
+        <v>98</v>
+      </c>
+      <c r="E47" t="s">
+        <v>211</v>
       </c>
       <c r="F47">
-        <v>9883106365</v>
-      </c>
-      <c r="G47" t="s">
-        <v>164</v>
+        <v>9830037452</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="B48">
-        <v>3516</v>
+        <v>11195</v>
       </c>
       <c r="C48" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D48" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="E48" t="s">
+        <v>140</v>
       </c>
       <c r="F48">
-        <v>9088321560</v>
-      </c>
-      <c r="G48" t="s">
-        <v>139</v>
+        <v>9330817822</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B49">
-        <v>165</v>
+        <v>19224</v>
       </c>
       <c r="C49" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D49" t="s">
-        <v>116</v>
-      </c>
-      <c r="F49">
-        <v>8697055924</v>
-      </c>
-      <c r="G49" t="s">
-        <v>165</v>
+        <v>97</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B50">
-        <v>120</v>
+        <v>165</v>
       </c>
       <c r="C50" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D50" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F50">
-        <v>6290999147</v>
-      </c>
-      <c r="G50" t="s">
-        <v>124</v>
+        <v>8697055924</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>55</v>
+        <v>213</v>
       </c>
       <c r="B51">
-        <v>10000</v>
+        <v>3516</v>
       </c>
       <c r="C51" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D51" t="s">
-        <v>117</v>
+        <v>96</v>
+      </c>
+      <c r="F51">
+        <v>9088321560</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="B52">
-        <v>7377</v>
+        <v>120</v>
       </c>
       <c r="C52" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D52" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F52">
-        <v>8777859764</v>
-      </c>
-      <c r="G52" t="s">
-        <v>166</v>
+        <v>6290999147</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="B53">
-        <v>16850</v>
+        <v>10000</v>
       </c>
       <c r="C53" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D53" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>58</v>
+        <v>214</v>
       </c>
       <c r="B54">
-        <v>1047</v>
+        <v>7377</v>
       </c>
       <c r="C54" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D54" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F54">
-        <v>9339111177</v>
-      </c>
-      <c r="G54" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+        <v>8777859764</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B55">
-        <v>16580</v>
+        <v>18200</v>
       </c>
       <c r="C55" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D55" t="s">
-        <v>117</v>
+        <v>97</v>
+      </c>
+      <c r="F55">
+        <v>9903404493</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>60</v>
+        <v>216</v>
       </c>
       <c r="B56">
-        <v>1881</v>
+        <v>1047</v>
       </c>
       <c r="C56" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D56" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F56">
-        <v>6290572487</v>
-      </c>
-      <c r="G56" t="s">
-        <v>168</v>
+        <v>9339111177</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>61</v>
+        <v>217</v>
       </c>
       <c r="B57">
-        <v>4990</v>
+        <v>1409</v>
       </c>
       <c r="C57" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D57" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F57">
-        <v>9674830246</v>
-      </c>
-      <c r="G57" t="s">
-        <v>169</v>
+        <v>9883106365</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B58">
-        <v>11514</v>
+        <v>16580</v>
       </c>
       <c r="C58" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D58" t="s">
-        <v>117</v>
-      </c>
-      <c r="F58">
-        <v>9883624996</v>
-      </c>
-      <c r="G58" t="s">
-        <v>151</v>
+        <v>97</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B59">
-        <v>5450</v>
+        <v>1881</v>
       </c>
       <c r="C59" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D59" t="s">
-        <v>116</v>
-      </c>
-      <c r="E59" t="s">
-        <v>170</v>
+        <v>96</v>
       </c>
       <c r="F59">
-        <v>9433276696</v>
-      </c>
-      <c r="G59" t="s">
-        <v>171</v>
+        <v>6290572487</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B60">
-        <v>631264.80000000005</v>
+        <v>4990</v>
       </c>
       <c r="C60" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D60" t="s">
-        <v>116</v>
-      </c>
-      <c r="E60" t="s">
-        <v>172</v>
+        <v>96</v>
       </c>
       <c r="F60">
-        <v>9830250558</v>
-      </c>
-      <c r="G60" t="s">
-        <v>173</v>
+        <v>9674830246</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B61">
-        <v>5100</v>
+        <v>15014</v>
       </c>
       <c r="C61" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D61" t="s">
-        <v>117</v>
-      </c>
-      <c r="E61" t="s">
-        <v>172</v>
+        <v>97</v>
       </c>
       <c r="F61">
-        <v>9830250558</v>
-      </c>
-      <c r="G61" t="s">
-        <v>173</v>
+        <v>9883624996</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="B62">
-        <v>11375</v>
+        <v>5450</v>
       </c>
       <c r="C62" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D62" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="E62" t="s">
-        <v>174</v>
+        <v>149</v>
       </c>
       <c r="F62">
+        <v>9433276696</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>52</v>
+      </c>
+      <c r="B63">
+        <v>621989</v>
+      </c>
+      <c r="C63" t="s">
+        <v>94</v>
+      </c>
+      <c r="D63" t="s">
+        <v>96</v>
+      </c>
+      <c r="E63" t="s">
+        <v>151</v>
+      </c>
+      <c r="F63">
+        <v>9830250558</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>53</v>
+      </c>
+      <c r="B64">
+        <v>36600</v>
+      </c>
+      <c r="C64" t="s">
+        <v>94</v>
+      </c>
+      <c r="D64" t="s">
+        <v>97</v>
+      </c>
+      <c r="E64" t="s">
+        <v>151</v>
+      </c>
+      <c r="F64">
+        <v>9830250558</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>54</v>
+      </c>
+      <c r="B65">
+        <v>9175</v>
+      </c>
+      <c r="C65" t="s">
+        <v>94</v>
+      </c>
+      <c r="D65" t="s">
+        <v>96</v>
+      </c>
+      <c r="E65" t="s">
+        <v>153</v>
+      </c>
+      <c r="F65">
         <v>9836772237</v>
       </c>
-      <c r="G62" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>67</v>
-      </c>
-      <c r="B63">
-        <v>10011</v>
-      </c>
-      <c r="C63" t="s">
-        <v>113</v>
-      </c>
-      <c r="D63" t="s">
-        <v>116</v>
-      </c>
-      <c r="E63" t="s">
-        <v>176</v>
-      </c>
-      <c r="F63">
+      <c r="G65" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>55</v>
+      </c>
+      <c r="B66">
+        <v>7366</v>
+      </c>
+      <c r="C66" t="s">
+        <v>94</v>
+      </c>
+      <c r="D66" t="s">
+        <v>96</v>
+      </c>
+      <c r="E66" t="s">
+        <v>155</v>
+      </c>
+      <c r="F66">
         <v>9836038802</v>
       </c>
-      <c r="G63" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>68</v>
-      </c>
-      <c r="B64">
+      <c r="G66" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>218</v>
+      </c>
+      <c r="B67">
         <v>15470</v>
       </c>
-      <c r="C64" t="s">
-        <v>113</v>
-      </c>
-      <c r="D64" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>69</v>
-      </c>
-      <c r="B65">
+      <c r="C67" t="s">
+        <v>94</v>
+      </c>
+      <c r="D67" t="s">
+        <v>96</v>
+      </c>
+      <c r="E67" t="s">
+        <v>219</v>
+      </c>
+      <c r="F67">
+        <v>9674100575</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>56</v>
+      </c>
+      <c r="B68">
         <v>21739</v>
       </c>
-      <c r="C65" t="s">
-        <v>113</v>
-      </c>
-      <c r="D65" t="s">
-        <v>116</v>
-      </c>
-      <c r="F65">
+      <c r="C68" t="s">
+        <v>94</v>
+      </c>
+      <c r="D68" t="s">
+        <v>96</v>
+      </c>
+      <c r="F68">
         <v>9874710290</v>
       </c>
-      <c r="G65" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>70</v>
-      </c>
-      <c r="B66">
-        <v>4495</v>
-      </c>
-      <c r="C66" t="s">
-        <v>113</v>
-      </c>
-      <c r="D66" t="s">
-        <v>117</v>
-      </c>
-      <c r="G66" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>71</v>
-      </c>
-      <c r="B67">
-        <v>40409</v>
-      </c>
-      <c r="C67" t="s">
-        <v>113</v>
-      </c>
-      <c r="D67" t="s">
-        <v>116</v>
-      </c>
-      <c r="F67">
-        <v>9903331444</v>
-      </c>
-      <c r="G67" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>72</v>
-      </c>
-      <c r="B68">
-        <v>8488</v>
-      </c>
-      <c r="C68" t="s">
-        <v>113</v>
-      </c>
-      <c r="D68" t="s">
-        <v>117</v>
-      </c>
-      <c r="F68">
-        <v>9674599644</v>
-      </c>
-      <c r="G68" t="s">
-        <v>180</v>
+      <c r="G68" s="3" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="B69">
-        <v>10760</v>
+        <v>40409</v>
       </c>
       <c r="C69" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D69" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F69">
-        <v>9883842122</v>
-      </c>
-      <c r="G69" t="s">
-        <v>139</v>
+        <v>9903331444</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B70">
-        <v>10545</v>
+        <v>6488</v>
       </c>
       <c r="C70" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D70" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="F70">
-        <v>8981612775</v>
-      </c>
-      <c r="G70" t="s">
-        <v>181</v>
+        <v>9674599644</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="B71">
-        <v>10615</v>
+        <v>28631.599999999999</v>
       </c>
       <c r="C71" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D71" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="F71">
+        <v>9883842122</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B72">
-        <v>42203</v>
+        <v>10545</v>
       </c>
       <c r="C72" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D72" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F72">
-        <v>6290829440</v>
-      </c>
-      <c r="G72" t="s">
-        <v>182</v>
+        <v>8981612775</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="B73">
-        <v>900</v>
+        <v>10615</v>
       </c>
       <c r="C73" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D73" t="s">
-        <v>116</v>
-      </c>
-      <c r="F73">
-        <v>6291105278</v>
-      </c>
-      <c r="G73" t="s">
-        <v>183</v>
+        <v>96</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="B74">
-        <v>35970</v>
+        <v>42203</v>
       </c>
       <c r="C74" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D74" t="s">
-        <v>117</v>
-      </c>
-      <c r="E74" t="s">
-        <v>184</v>
+        <v>96</v>
       </c>
       <c r="F74">
-        <v>9748216805</v>
-      </c>
-      <c r="G74" t="s">
-        <v>185</v>
+        <v>6290829440</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="B75">
-        <v>57920</v>
+        <v>900</v>
       </c>
       <c r="C75" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D75" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F75">
-        <v>9051261192</v>
-      </c>
-      <c r="G75" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+        <v>6291105278</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="B76">
-        <v>36636</v>
+        <v>36970</v>
       </c>
       <c r="C76" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D76" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="E76" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="F76">
         <v>9748216805</v>
       </c>
-      <c r="G76" t="s">
-        <v>185</v>
+      <c r="G76" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>81</v>
+        <v>221</v>
       </c>
       <c r="B77">
-        <v>33950</v>
+        <v>57420</v>
       </c>
       <c r="C77" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D77" t="s">
-        <v>117</v>
-      </c>
-      <c r="E77" t="s">
-        <v>187</v>
+        <v>96</v>
       </c>
       <c r="F77">
-        <v>9775229565</v>
-      </c>
-      <c r="G77" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+        <v>9051261192</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>82</v>
+        <v>65</v>
       </c>
       <c r="B78">
-        <v>3186</v>
+        <v>32636</v>
       </c>
       <c r="C78" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D78" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="E78" t="s">
+        <v>163</v>
       </c>
       <c r="F78">
-        <v>8420464321</v>
-      </c>
-      <c r="G78" t="s">
-        <v>139</v>
+        <v>9748216805</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="B79">
-        <v>0</v>
+        <v>33950</v>
       </c>
       <c r="C79" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="D79" t="s">
-        <v>119</v>
+        <v>97</v>
       </c>
       <c r="E79" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="F79">
-        <v>8583811502</v>
-      </c>
-      <c r="G79" t="s">
-        <v>190</v>
+        <v>9775229565</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="B80">
-        <v>9045</v>
+        <v>3186</v>
       </c>
       <c r="C80" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D80" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="F80">
-        <v>9062188967</v>
-      </c>
-      <c r="G80" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+        <v>8420464321</v>
+      </c>
+      <c r="G80" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>115</v>
+        <v>68</v>
       </c>
       <c r="B81">
-        <v>13957</v>
+        <v>0</v>
       </c>
       <c r="C81" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D81" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="E81" t="s">
+        <v>168</v>
+      </c>
+      <c r="F81">
+        <v>8583811502</v>
+      </c>
+      <c r="G81" s="3" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>85</v>
+        <v>222</v>
       </c>
       <c r="B82">
-        <v>1283</v>
+        <v>9025</v>
       </c>
       <c r="C82" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D82" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="F82">
-        <v>9433128455</v>
-      </c>
-      <c r="G82" t="s">
-        <v>167</v>
+        <v>9062188967</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>86</v>
+        <v>223</v>
       </c>
       <c r="B83">
-        <v>7271</v>
+        <v>13957</v>
       </c>
       <c r="C83" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D83" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F83">
-        <v>9330849331</v>
-      </c>
-      <c r="G83" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+        <v>9331834709</v>
+      </c>
+      <c r="G83" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>87</v>
+        <v>224</v>
       </c>
       <c r="B84">
-        <v>1924</v>
+        <v>0</v>
       </c>
       <c r="C84" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D84" t="s">
-        <v>116</v>
+        <v>98</v>
+      </c>
+      <c r="E84" t="s">
+        <v>225</v>
       </c>
       <c r="F84">
-        <v>9038307447</v>
+        <v>8648923453</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="B85">
-        <v>0</v>
+        <v>1283</v>
       </c>
       <c r="C85" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D85" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="F85">
+        <v>9433128455</v>
+      </c>
+      <c r="G85" s="3" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="B86">
-        <v>13795</v>
+        <v>7271</v>
       </c>
       <c r="C86" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D86" t="s">
-        <v>117</v>
-      </c>
-      <c r="E86" t="s">
-        <v>193</v>
+        <v>96</v>
       </c>
       <c r="F86">
-        <v>9874372584</v>
-      </c>
-      <c r="G86" t="s">
-        <v>194</v>
+        <v>9330849331</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>90</v>
+        <v>227</v>
       </c>
       <c r="B87">
-        <v>7799</v>
+        <v>0</v>
       </c>
       <c r="C87" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D87" t="s">
-        <v>116</v>
+        <v>237</v>
+      </c>
+      <c r="E87" t="s">
+        <v>228</v>
       </c>
       <c r="F87">
-        <v>9748966299</v>
-      </c>
-      <c r="G87" t="s">
-        <v>195</v>
+        <v>9831044239</v>
+      </c>
+      <c r="G87" s="3" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="B88">
-        <v>3050</v>
+        <v>4114</v>
       </c>
       <c r="C88" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D88" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="F88">
+        <v>9038307447</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="B89">
-        <v>38572</v>
+        <v>0</v>
       </c>
       <c r="C89" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D89" t="s">
-        <v>116</v>
-      </c>
-      <c r="G89" t="s">
-        <v>129</v>
+        <v>96</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>93</v>
+        <v>230</v>
       </c>
       <c r="B90">
-        <v>5350</v>
+        <v>13795</v>
       </c>
       <c r="C90" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D90" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="E90" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="F90">
-        <v>9062449752</v>
-      </c>
-      <c r="G90" t="s">
-        <v>197</v>
+        <v>9874372584</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>94</v>
+        <v>231</v>
       </c>
       <c r="B91">
-        <v>30462</v>
+        <v>7799</v>
       </c>
       <c r="C91" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D91" t="s">
-        <v>117</v>
-      </c>
-      <c r="G91" t="s">
-        <v>198</v>
+        <v>96</v>
+      </c>
+      <c r="F91">
+        <v>9748966299</v>
+      </c>
+      <c r="G91" s="3" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>95</v>
+        <v>73</v>
       </c>
       <c r="B92">
-        <v>4441</v>
+        <v>3050</v>
       </c>
       <c r="C92" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D92" t="s">
-        <v>116</v>
-      </c>
-      <c r="G92" t="s">
-        <v>129</v>
+        <v>96</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="B93">
-        <v>4218</v>
+        <v>38572</v>
       </c>
       <c r="C93" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D93" t="s">
-        <v>117</v>
-      </c>
-      <c r="F93">
-        <v>8420333152</v>
-      </c>
-      <c r="G93" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+      <c r="G93" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>97</v>
+        <v>75</v>
       </c>
       <c r="B94">
-        <v>191150</v>
+        <v>5350</v>
       </c>
       <c r="C94" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D94" t="s">
-        <v>117</v>
-      </c>
-      <c r="G94" t="s">
-        <v>200</v>
+        <v>96</v>
+      </c>
+      <c r="E94" t="s">
+        <v>175</v>
+      </c>
+      <c r="F94">
+        <v>9062449752</v>
+      </c>
+      <c r="G94" s="3" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="B95">
-        <v>37324</v>
+        <v>20562</v>
       </c>
       <c r="C95" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D95" t="s">
-        <v>117</v>
-      </c>
-      <c r="E95" t="s">
-        <v>201</v>
-      </c>
-      <c r="F95">
-        <v>9163123281</v>
-      </c>
-      <c r="G95" t="s">
-        <v>202</v>
+        <v>97</v>
+      </c>
+      <c r="G95" s="3" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="B96">
-        <v>23506</v>
+        <v>4441</v>
       </c>
       <c r="C96" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D96" t="s">
-        <v>116</v>
-      </c>
-      <c r="F96">
-        <v>9331098987</v>
-      </c>
-      <c r="G96" t="s">
-        <v>203</v>
+        <v>96</v>
+      </c>
+      <c r="G96" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="B97">
-        <v>5865</v>
+        <v>4218</v>
       </c>
       <c r="C97" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D97" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F97">
-        <v>7003928847</v>
-      </c>
-      <c r="G97" t="s">
-        <v>204</v>
+        <v>8420333152</v>
+      </c>
+      <c r="G97" s="3" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>101</v>
+        <v>232</v>
       </c>
       <c r="B98">
-        <v>18615</v>
+        <v>99457</v>
       </c>
       <c r="C98" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D98" t="s">
-        <v>117</v>
-      </c>
-      <c r="E98" t="s">
-        <v>205</v>
+        <v>97</v>
       </c>
       <c r="F98">
-        <v>8910875876</v>
-      </c>
-      <c r="G98" t="s">
-        <v>206</v>
+        <v>7439001310</v>
+      </c>
+      <c r="G98" s="3" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="B99">
-        <v>42193</v>
+        <v>44049</v>
       </c>
       <c r="C99" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D99" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="E99" t="s">
-        <v>207</v>
+        <v>179</v>
       </c>
       <c r="F99">
-        <v>9382319739</v>
-      </c>
-      <c r="G99" t="s">
-        <v>208</v>
+        <v>9163123281</v>
+      </c>
+      <c r="G99" s="3" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="B100">
-        <v>2000</v>
+        <v>26744</v>
       </c>
       <c r="C100" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D100" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F100">
-        <v>7059704884</v>
-      </c>
-      <c r="G100" t="s">
-        <v>151</v>
+        <v>9331098987</v>
+      </c>
+      <c r="G100" s="3" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="B101">
-        <v>1700</v>
+        <v>5865</v>
       </c>
       <c r="C101" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D101" t="s">
-        <v>116</v>
+        <v>96</v>
       </c>
       <c r="F101">
-        <v>9681297975</v>
-      </c>
-      <c r="G101" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+        <v>7003928847</v>
+      </c>
+      <c r="G101" s="3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="B102">
-        <v>6126</v>
+        <v>20115</v>
       </c>
       <c r="C102" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D102" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="E102" t="s">
+        <v>183</v>
       </c>
       <c r="F102">
-        <v>8777286730</v>
-      </c>
-      <c r="G102" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+        <v>8910875876</v>
+      </c>
+      <c r="G102" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="B103">
-        <v>5128</v>
+        <v>42193</v>
       </c>
       <c r="C103" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D103" t="s">
-        <v>116</v>
+        <v>96</v>
+      </c>
+      <c r="E103" t="s">
+        <v>185</v>
       </c>
       <c r="F103">
-        <v>9874398875</v>
-      </c>
-      <c r="G103" t="s">
-        <v>211</v>
+        <v>9382319739</v>
+      </c>
+      <c r="G103" s="3" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="B104">
-        <v>750</v>
+        <v>2000</v>
       </c>
       <c r="C104" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D104" t="s">
-        <v>116</v>
-      </c>
-      <c r="G104" t="s">
-        <v>129</v>
+        <v>96</v>
+      </c>
+      <c r="F104">
+        <v>7059704884</v>
+      </c>
+      <c r="G104" s="3" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="B105">
-        <v>34068</v>
+        <v>1700</v>
       </c>
       <c r="C105" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="D105" t="s">
-        <v>117</v>
-      </c>
-      <c r="E105" t="s">
-        <v>212</v>
+        <v>96</v>
       </c>
       <c r="F105">
-        <v>9874776367</v>
-      </c>
-      <c r="G105" t="s">
-        <v>213</v>
+        <v>9681297975</v>
+      </c>
+      <c r="G105" s="3" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>109</v>
+        <v>86</v>
       </c>
       <c r="B106">
-        <v>3920</v>
+        <v>6126</v>
       </c>
       <c r="C106" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D106" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="F106">
-        <v>9330953545</v>
-      </c>
-      <c r="G106" t="s">
-        <v>214</v>
+        <v>8777286730</v>
+      </c>
+      <c r="G106" s="3" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="B107">
-        <v>46695</v>
+        <v>5128</v>
       </c>
       <c r="C107" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D107" t="s">
-        <v>117</v>
+        <v>96</v>
+      </c>
+      <c r="F107">
+        <v>9874398875</v>
+      </c>
+      <c r="G107" s="3" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="B108">
-        <v>27356</v>
+        <v>750</v>
       </c>
       <c r="C108" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="D108" t="s">
-        <v>117</v>
-      </c>
-      <c r="E108" t="s">
-        <v>215</v>
-      </c>
-      <c r="G108" t="s">
-        <v>216</v>
+        <v>96</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>89</v>
+      </c>
+      <c r="B109">
+        <v>35278</v>
+      </c>
+      <c r="C109" t="s">
+        <v>94</v>
+      </c>
+      <c r="D109" t="s">
+        <v>97</v>
+      </c>
+      <c r="E109" t="s">
+        <v>190</v>
+      </c>
+      <c r="F109">
+        <v>9874776367</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>234</v>
+      </c>
+      <c r="B110">
+        <v>52497</v>
+      </c>
+      <c r="C110" t="s">
+        <v>94</v>
+      </c>
+      <c r="D110" t="s">
+        <v>97</v>
+      </c>
+      <c r="E110" t="s">
+        <v>235</v>
+      </c>
+      <c r="F110">
+        <v>7003428106</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>90</v>
+      </c>
+      <c r="B111">
+        <v>1420</v>
+      </c>
+      <c r="C111" t="s">
+        <v>94</v>
+      </c>
+      <c r="D111" t="s">
+        <v>97</v>
+      </c>
+      <c r="F111">
+        <v>9330953545</v>
+      </c>
+      <c r="G111" s="3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>91</v>
+      </c>
+      <c r="B112">
+        <v>0</v>
+      </c>
+      <c r="C112" t="s">
+        <v>94</v>
+      </c>
+      <c r="D112" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>92</v>
+      </c>
+      <c r="B113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="s">
+        <v>94</v>
+      </c>
+      <c r="D113" t="s">
+        <v>97</v>
+      </c>
+      <c r="E113" t="s">
+        <v>193</v>
+      </c>
+      <c r="G113" s="3" t="s">
+        <v>194</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G108" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>